<commit_message>
Corrida | SFE-VTTR | 2026-05-08 09:59:55.05368
</commit_message>
<xml_diff>
--- a/indicadores/SFE-VTTR_out.xlsx
+++ b/indicadores/SFE-VTTR_out.xlsx
@@ -104,13 +104,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">07/05/2026</t>
+    <t xml:space="preserve">08/05/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">ysonder</t>
+    <t xml:space="preserve">pcohan</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>

</xml_diff>